<commit_message>
Add RBO scores and remove obsolete Excel file.
</commit_message>
<xml_diff>
--- a/Graph_v2/comparing graph v1 x v2.xlsx
+++ b/Graph_v2/comparing graph v1 x v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOUTORADO\units\XAI4Spectra\Graph_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80EAAEEF-250F-4F39-97A2-E59F87CD3F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B22825-41BB-44FD-9A9E-4114BE6C3209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{377E04CD-142B-42C0-B4DA-AF18741D1B3A}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="soil BSP" sheetId="2" r:id="rId2"/>
     <sheet name="synthetic" sheetId="3" r:id="rId3"/>
     <sheet name="soil types" sheetId="4" r:id="rId4"/>
+    <sheet name="milk" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="67">
   <si>
     <t>Vip</t>
   </si>
@@ -211,6 +212,33 @@
   </si>
   <si>
     <t>metric</t>
+  </si>
+  <si>
+    <t>Ag La</t>
+  </si>
+  <si>
+    <t>Ag ka</t>
+  </si>
+  <si>
+    <t>Ag Lb</t>
+  </si>
+  <si>
+    <t>Zn</t>
+  </si>
+  <si>
+    <t>Fe</t>
+  </si>
+  <si>
+    <t>Bremsstrahlung</t>
+  </si>
+  <si>
+    <t>Ag compton</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>background</t>
   </si>
 </sst>
 </file>
@@ -226,7 +254,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -245,6 +273,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -258,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -275,22 +309,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,15 +660,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="9"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7" t="s">
+      <c r="E1" s="10"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="7"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -648,13 +686,13 @@
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>50</v>
       </c>
       <c r="J2" s="1" t="s">
@@ -684,13 +722,13 @@
       <c r="E3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -699,7 +737,7 @@
       <c r="K3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="9">
         <v>0.922268771763333</v>
       </c>
       <c r="M3" s="1" t="s">
@@ -722,13 +760,13 @@
       <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="1" t="s">
@@ -737,7 +775,7 @@
       <c r="K4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="9">
         <v>0.87326877176333295</v>
       </c>
       <c r="M4" s="1" t="s">
@@ -760,13 +798,13 @@
       <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="J5" s="1" t="s">
@@ -775,7 +813,7 @@
       <c r="K5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <v>0.46280367730333299</v>
       </c>
       <c r="M5" s="1" t="s">
@@ -798,13 +836,13 @@
       <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>9</v>
       </c>
       <c r="J6" s="1" t="s">
@@ -813,7 +851,7 @@
       <c r="K6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="9">
         <v>0.44955188030666599</v>
       </c>
       <c r="M6" s="1" t="s">
@@ -836,13 +874,13 @@
       <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="J7" s="1" t="s">
@@ -851,7 +889,7 @@
       <c r="K7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="9">
         <v>0.33014588030666597</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -874,13 +912,13 @@
       <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J8" s="1" t="s">
@@ -889,7 +927,7 @@
       <c r="K8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="9">
         <v>0.23575478551333301</v>
       </c>
       <c r="M8" s="1" t="s">
@@ -912,13 +950,13 @@
       <c r="E9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>12</v>
       </c>
       <c r="J9" s="1" t="s">
@@ -927,7 +965,7 @@
       <c r="K9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="9">
         <v>0.206953982176666</v>
       </c>
       <c r="M9" s="1" t="s">
@@ -950,13 +988,13 @@
       <c r="E10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -976,13 +1014,13 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1002,13 +1040,13 @@
       <c r="E12" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1028,13 +1066,13 @@
       <c r="E13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1054,13 +1092,13 @@
       <c r="E14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1080,13 +1118,13 @@
       <c r="E15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1106,13 +1144,13 @@
       <c r="E16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="6" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1132,13 +1170,13 @@
       <c r="E17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1158,13 +1196,13 @@
       <c r="E18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="6" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1184,13 +1222,13 @@
       <c r="E19" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="6" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1210,13 +1248,13 @@
       <c r="E20" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="7" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1254,9 +1292,9 @@
     <col min="1" max="3" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.88671875" style="2"/>
     <col min="10" max="10" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1265,11 +1303,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="9"/>
-      <c r="G1" s="7" t="s">
+      <c r="E1" s="10"/>
+      <c r="G1" s="6" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1289,13 +1327,13 @@
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>50</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -1324,13 +1362,13 @@
       <c r="E3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>7</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -1339,7 +1377,7 @@
       <c r="K3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="9">
         <v>0.91891908064000005</v>
       </c>
       <c r="M3" s="1" t="s">
@@ -1362,13 +1400,13 @@
       <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>27</v>
       </c>
       <c r="J4" s="1" t="s">
@@ -1377,7 +1415,7 @@
       <c r="K4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="9">
         <v>0.79400548063999898</v>
       </c>
       <c r="M4" s="1" t="s">
@@ -1400,13 +1438,13 @@
       <c r="E5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J5" s="1" t="s">
@@ -1415,7 +1453,7 @@
       <c r="K5" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <v>0.79208388030666599</v>
       </c>
       <c r="M5" s="1" t="s">
@@ -1438,13 +1476,13 @@
       <c r="E6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J6" s="1" t="s">
@@ -1453,7 +1491,7 @@
       <c r="K6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="9">
         <v>0.78656928030666595</v>
       </c>
       <c r="M6" s="1" t="s">
@@ -1476,13 +1514,13 @@
       <c r="E7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J7" s="1" t="s">
@@ -1491,7 +1529,7 @@
       <c r="K7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="9">
         <v>0.78246977209666602</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -1514,13 +1552,13 @@
       <c r="E8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="J8" s="1" t="s">
@@ -1529,7 +1567,7 @@
       <c r="K8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="9">
         <v>0.65927787396666604</v>
       </c>
       <c r="M8" s="1" t="s">
@@ -1552,13 +1590,13 @@
       <c r="E9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J9" s="1" t="s">
@@ -1567,7 +1605,7 @@
       <c r="K9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="9">
         <v>0.32916446355333301</v>
       </c>
       <c r="M9" s="1" t="s">
@@ -1590,16 +1628,16 @@
       <c r="E10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="L10" s="11"/>
+      <c r="L10" s="9"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -1617,13 +1655,13 @@
       <c r="E11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1643,13 +1681,13 @@
       <c r="E12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1669,13 +1707,13 @@
       <c r="E13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1695,13 +1733,13 @@
       <c r="E14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="6" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1721,13 +1759,13 @@
       <c r="E15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="6" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1747,13 +1785,13 @@
       <c r="E16" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="6" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1773,13 +1811,13 @@
       <c r="E17" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="6" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1799,13 +1837,13 @@
       <c r="E18" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1825,13 +1863,13 @@
       <c r="E19" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="6" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1851,13 +1889,13 @@
       <c r="E20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="6" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1877,13 +1915,13 @@
       <c r="E21" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" s="6" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1903,13 +1941,13 @@
       <c r="E22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="6" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1929,13 +1967,13 @@
       <c r="E23" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="6" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1955,13 +1993,13 @@
       <c r="E24" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1981,13 +2019,13 @@
       <c r="E25" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="6" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2007,13 +2045,13 @@
       <c r="E26" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2033,13 +2071,13 @@
       <c r="E27" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H27" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2059,13 +2097,13 @@
       <c r="E28" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="6" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2082,10 +2120,10 @@
       <c r="D29" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2102,10 +2140,10 @@
       <c r="D30" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2122,10 +2160,10 @@
       <c r="D31" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="G31" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="H31" s="6" t="s">
         <v>22</v>
       </c>
     </row>
@@ -2142,10 +2180,10 @@
       <c r="D32" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G32" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H32" s="6" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2179,15 +2217,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="8"/>
       <c r="M1" s="2"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2206,13 +2244,13 @@
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="8" t="s">
         <v>50</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -2242,13 +2280,13 @@
       <c r="E3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -2280,13 +2318,13 @@
       <c r="E4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="8" t="s">
         <v>45</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -2318,13 +2356,13 @@
       <c r="E5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="8" t="s">
         <v>46</v>
       </c>
       <c r="J5" s="2" t="s">
@@ -2356,13 +2394,13 @@
       <c r="E6" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="8" t="s">
         <v>16</v>
       </c>
       <c r="J6" s="2" t="s">
@@ -2394,13 +2432,13 @@
       <c r="E7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J7" s="2" t="s">
@@ -2432,13 +2470,13 @@
       <c r="E8" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="8" t="s">
         <v>47</v>
       </c>
       <c r="J8" s="2" t="s">
@@ -2470,13 +2508,13 @@
       <c r="E9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="8" t="s">
         <v>48</v>
       </c>
       <c r="J9" s="2" t="s">
@@ -2508,13 +2546,13 @@
       <c r="E10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="8" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2534,13 +2572,13 @@
       <c r="E11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2560,13 +2598,13 @@
       <c r="E12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="8" t="s">
         <v>22</v>
       </c>
     </row>
@@ -2584,11 +2622,11 @@
         <v>20</v>
       </c>
       <c r="E13" s="5"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10" t="s">
+      <c r="F13" s="8"/>
+      <c r="G13" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2606,11 +2644,11 @@
         <v>18</v>
       </c>
       <c r="E14" s="5"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10" t="s">
+      <c r="F14" s="8"/>
+      <c r="G14" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="8" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2645,15 +2683,15 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C1" s="1"/>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="10"/>
+      <c r="H1" s="8"/>
       <c r="M1" s="2"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2672,13 +2710,13 @@
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="8" t="s">
         <v>50</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -2708,13 +2746,13 @@
       <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="7" t="s">
         <v>7</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -2746,13 +2784,13 @@
       <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="7" t="s">
         <v>5</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -2784,13 +2822,13 @@
       <c r="E5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>6</v>
       </c>
       <c r="J5" s="2" t="s">
@@ -2822,13 +2860,13 @@
       <c r="E6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="J6" s="2" t="s">
@@ -2860,13 +2898,13 @@
       <c r="E7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>27</v>
       </c>
       <c r="J7" s="2" t="s">
@@ -2898,13 +2936,13 @@
       <c r="E8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="J8" s="2" t="s">
@@ -2936,13 +2974,13 @@
       <c r="E9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="J9" s="2" t="s">
@@ -2974,13 +3012,13 @@
       <c r="E10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3000,13 +3038,13 @@
       <c r="E11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="7" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3026,13 +3064,13 @@
       <c r="E12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3052,13 +3090,13 @@
       <c r="E13" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="7" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3078,13 +3116,13 @@
       <c r="E14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="7" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3104,13 +3142,13 @@
       <c r="E15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -3130,13 +3168,13 @@
       <c r="E16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3156,13 +3194,13 @@
       <c r="E17" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="H17" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3182,13 +3220,13 @@
       <c r="E18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3208,13 +3246,13 @@
       <c r="E19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="7" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3234,13 +3272,13 @@
       <c r="E20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3260,13 +3298,13 @@
       <c r="E21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3286,13 +3324,13 @@
       <c r="E22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="7" t="s">
         <v>22</v>
       </c>
     </row>
@@ -3312,13 +3350,13 @@
       <c r="E23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="7" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3338,13 +3376,13 @@
       <c r="E24" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="H24" s="7" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3364,13 +3402,13 @@
       <c r="E25" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="7" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3390,13 +3428,13 @@
       <c r="E26" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="H26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3414,11 +3452,11 @@
         <v>20</v>
       </c>
       <c r="E27" s="4"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8" t="s">
+      <c r="F27" s="7"/>
+      <c r="G27" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="H27" s="7" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3431,4 +3469,263 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F555155F-3C70-4D5C-90FD-27CD346F93A8}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.96478877476666602</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0.86366418884999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.81512968885000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.36421797509999898</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove unused code blocks from the project.
</commit_message>
<xml_diff>
--- a/Graph_v2/comparing graph v1 x v2.xlsx
+++ b/Graph_v2/comparing graph v1 x v2.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOUTORADO\units\XAI4Spectra\Graph_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B22825-41BB-44FD-9A9E-4114BE6C3209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5680A6D8-2EAE-411E-8A53-45B46DF8558F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{377E04CD-142B-42C0-B4DA-AF18741D1B3A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{377E04CD-142B-42C0-B4DA-AF18741D1B3A}"/>
   </bookViews>
   <sheets>
-    <sheet name="bank_notes" sheetId="1" r:id="rId1"/>
-    <sheet name="soil BSP" sheetId="2" r:id="rId2"/>
-    <sheet name="synthetic" sheetId="3" r:id="rId3"/>
+    <sheet name="synthetic" sheetId="3" r:id="rId1"/>
+    <sheet name="bank_notes" sheetId="1" r:id="rId2"/>
+    <sheet name="soil BSP" sheetId="2" r:id="rId3"/>
     <sheet name="soil types" sheetId="4" r:id="rId4"/>
     <sheet name="milk" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -319,6 +319,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -328,7 +329,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -642,6 +642,471 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F68501-B4CF-4069-8217-47030F8915B3}">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="11.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="14.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="12"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="M1" s="2"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0.97175247509999996</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0.95734647509999904</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.92540098030666595</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0.92321797510000003</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L7" s="3">
+        <v>0.91845358063999905</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" s="3">
+        <v>0.87640098030666602</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" s="3">
+        <v>0.71113838551333297</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J3:M9">
+    <sortCondition descending="1" ref="L3:L9"/>
+  </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1432A4DF-60D1-470F-8CA8-3C816860528C}">
   <dimension ref="A1:M28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -660,10 +1125,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="10"/>
+      <c r="E1" s="11"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6" t="s">
         <v>54</v>
@@ -1284,7 +1749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E6FC434-47C9-451A-BC52-87804B6B0492}">
   <dimension ref="A1:M32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1303,10 +1768,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="10"/>
+      <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
         <v>54</v>
       </c>
@@ -2185,471 +2650,6 @@
       </c>
       <c r="H32" s="6" t="s">
         <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J3:M9">
-    <sortCondition descending="1" ref="L3:L9"/>
-  </sortState>
-  <mergeCells count="1">
-    <mergeCell ref="D1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F68501-B4CF-4069-8217-47030F8915B3}">
-  <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="11.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="14.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.88671875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D1" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="11"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="8"/>
-      <c r="M1" s="2"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0.97175247509999996</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="3">
-        <v>0.95734647509999904</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="L5" s="3">
-        <v>0.92540098030666595</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L6" s="3">
-        <v>0.92321797510000003</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="L7" s="3">
-        <v>0.91845358063999905</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="L8" s="3">
-        <v>0.87640098030666602</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L9" s="3">
-        <v>0.71113838551333297</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2683,10 +2683,10 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C1" s="1"/>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="11"/>
+      <c r="E1" s="12"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8" t="s">
         <v>54</v>
@@ -3485,10 +3485,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="12"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -3500,10 +3500,10 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -3526,10 +3526,10 @@
       <c r="C3" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="10" t="s">
         <v>58</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -3552,10 +3552,10 @@
       <c r="C4" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>60</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -3578,10 +3578,10 @@
       <c r="C5" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="10" t="s">
         <v>59</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -3604,10 +3604,10 @@
       <c r="C6" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="10" t="s">
         <v>61</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -3630,10 +3630,10 @@
       <c r="C7" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="10" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3647,10 +3647,10 @@
       <c r="C8" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3664,10 +3664,10 @@
       <c r="C9" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="10" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3681,10 +3681,10 @@
       <c r="C10" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3698,10 +3698,10 @@
       <c r="C11" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="10" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3715,10 +3715,10 @@
       <c r="C12" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="10" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>